<commit_message>
ATUALIZAÇÃO DO COD DO ROLAMENTO
</commit_message>
<xml_diff>
--- a/dados-catalago-pcm-interno/nomes_usuais.xlsx
+++ b/dados-catalago-pcm-interno/nomes_usuais.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://amaggicombr-my.sharepoint.com/personal/hiago_andre_amaggi_com_br/Documents/Área de Trabalho/codigos/catalogoPecasPCM/dados-catalago-pcm-interno/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="197" documentId="11_AD4D361C20488DEA4E38A03414D973025ADEDD81" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5349278A-4B39-443E-9976-97319790B4FC}"/>
+  <xr:revisionPtr revIDLastSave="198" documentId="11_AD4D361C20488DEA4E38A03414D973025ADEDD81" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D1F792B3-8E27-4F0E-B05E-AA3A495EA65D}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
@@ -5254,8 +5254,8 @@
       </c>
     </row>
     <row r="286" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A286" s="15">
-        <v>1040098437</v>
+      <c r="A286" s="5">
+        <v>1040100107</v>
       </c>
       <c r="B286" s="5" t="s">
         <v>271</v>

</xml_diff>